<commit_message>
Actualizacion automatica de datos Asana y KPI 2026-06-18 19:12 UTC
</commit_message>
<xml_diff>
--- a/data/50001498 - CALABRESSE METRO STO DOMINGO POZOS.xlsx
+++ b/data/50001498 - CALABRESSE METRO STO DOMINGO POZOS.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1002" uniqueCount="289">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1004" uniqueCount="289">
   <si>
     <t xml:space="preserve">50001498-CALABRESSE METRO STO DOMINGO  POZOS  </t>
   </si>
@@ -583,70 +583,70 @@
     <t>Control de calidad compras materiales a codigo // compras locale aprovisionamiento,Bodega:,Bodega:</t>
   </si>
   <si>
+    <t>1213380470331436</t>
+  </si>
+  <si>
+    <t>Control de calidad compras materiales a codigo // compras locale aprovisionamiento</t>
+  </si>
+  <si>
+    <t>Nicolás López</t>
+  </si>
+  <si>
+    <t>nicolas.lopez@zitron.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bodega:,Generacion OC Fabricación externa </t>
+  </si>
+  <si>
+    <t>1213380470331437</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fabricación externa </t>
+  </si>
+  <si>
+    <t>Generacion OC Fabricación externa ,Armado fabricación externa ,Control de calidad Armado</t>
+  </si>
+  <si>
+    <t>1213380470331438</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Generacion OC Fabricación externa </t>
+  </si>
+  <si>
+    <t>Rosemary Singh</t>
+  </si>
+  <si>
+    <t>rosemary.singh@zitron.com</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Armado fabricación externa ,Fabricación externa </t>
+  </si>
+  <si>
+    <t>1213380470331439</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Armado fabricación externa </t>
+  </si>
+  <si>
+    <t>Generacion OC Fabricación externa ,Check Planos</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Control de calidad Armado,Fabricación externa </t>
+  </si>
+  <si>
+    <t>1213380470331440</t>
+  </si>
+  <si>
+    <t>Control de calidad Armado</t>
+  </si>
+  <si>
+    <t>Armado fabricación externa ,Check Planos</t>
+  </si>
+  <si>
+    <t>Fabricación externa ,Revestimiento</t>
+  </si>
+  <si>
     <t>Tarea en curso</t>
-  </si>
-  <si>
-    <t>1213380470331436</t>
-  </si>
-  <si>
-    <t>Control de calidad compras materiales a codigo // compras locale aprovisionamiento</t>
-  </si>
-  <si>
-    <t>Nicolás López</t>
-  </si>
-  <si>
-    <t>nicolas.lopez@zitron.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Bodega:,Generacion OC Fabricación externa </t>
-  </si>
-  <si>
-    <t>1213380470331437</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Fabricación externa </t>
-  </si>
-  <si>
-    <t>Generacion OC Fabricación externa ,Armado fabricación externa ,Control de calidad Armado</t>
-  </si>
-  <si>
-    <t>1213380470331438</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Generacion OC Fabricación externa </t>
-  </si>
-  <si>
-    <t>Rosemary Singh</t>
-  </si>
-  <si>
-    <t>rosemary.singh@zitron.com</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Armado fabricación externa ,Fabricación externa </t>
-  </si>
-  <si>
-    <t>1213380470331439</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Armado fabricación externa </t>
-  </si>
-  <si>
-    <t>Generacion OC Fabricación externa ,Check Planos</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Control de calidad Armado,Fabricación externa </t>
-  </si>
-  <si>
-    <t>1213380470331440</t>
-  </si>
-  <si>
-    <t>Control de calidad Armado</t>
-  </si>
-  <si>
-    <t>Armado fabricación externa ,Check Planos</t>
-  </si>
-  <si>
-    <t>Fabricación externa ,Revestimiento</t>
   </si>
   <si>
     <t>1213380470331441</t>
@@ -4336,9 +4336,11 @@
       <c r="B50" s="5">
         <v>46073.71759030093</v>
       </c>
-      <c r="C50" s="6"/>
+      <c r="C50" s="5">
+        <v>46191.78929271991</v>
+      </c>
       <c r="D50" s="5">
-        <v>46083.66881403935</v>
+        <v>46191.789304328704</v>
       </c>
       <c r="E50" s="6" t="s">
         <v>184</v>
@@ -4372,9 +4374,13 @@
       </c>
       <c r="Q50" s="6"/>
       <c r="R50" s="6"/>
-      <c r="S50" s="6"/>
+      <c r="S50" s="6">
+        <v>1</v>
+      </c>
       <c r="T50" s="6"/>
-      <c r="U50" s="6"/>
+      <c r="U50" s="11" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A51" s="7" t="s">
@@ -4383,9 +4389,11 @@
       <c r="B51" s="8">
         <v>46073.7175905787</v>
       </c>
-      <c r="C51" s="9"/>
+      <c r="C51" s="8">
+        <v>46191.788401875005</v>
+      </c>
       <c r="D51" s="8">
-        <v>46182.53061851852</v>
+        <v>46191.788422488426</v>
       </c>
       <c r="E51" s="9" t="s">
         <v>163</v>
@@ -4430,37 +4438,39 @@
         <v>46070</v>
       </c>
       <c r="S51" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T51" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="U51" s="12" t="s">
-        <v>190</v>
+      <c r="U51" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A52" s="4" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B52" s="5">
         <v>46073.717590810185</v>
       </c>
-      <c r="C52" s="6"/>
+      <c r="C52" s="5">
+        <v>46191.78927659722</v>
+      </c>
       <c r="D52" s="5">
-        <v>46091.742591689814</v>
+        <v>46191.789293194444</v>
       </c>
       <c r="E52" s="6" t="s">
+        <v>191</v>
+      </c>
+      <c r="F52" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G52" s="6" t="s">
         <v>192</v>
       </c>
-      <c r="F52" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G52" s="6" t="s">
+      <c r="H52" s="6" t="s">
         <v>193</v>
-      </c>
-      <c r="H52" s="6" t="s">
-        <v>194</v>
       </c>
       <c r="I52" s="5">
         <v>46071</v>
@@ -4484,7 +4494,7 @@
         <v>163</v>
       </c>
       <c r="P52" s="6" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="Q52" s="5">
         <v>46071</v>
@@ -4493,28 +4503,30 @@
         <v>46072</v>
       </c>
       <c r="S52" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T52" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="U52" s="10" t="s">
-        <v>56</v>
+      <c r="U52" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="53" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A53" s="7" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B53" s="8">
         <v>46073.717591099536</v>
       </c>
-      <c r="C53" s="9"/>
+      <c r="C53" s="8">
+        <v>46191.79037481482</v>
+      </c>
       <c r="D53" s="8">
-        <v>46129.78275488426</v>
+        <v>46191.79038505787</v>
       </c>
       <c r="E53" s="9" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="F53" s="9" t="s">
         <v>25</v>
@@ -4538,39 +4550,45 @@
         <v>26</v>
       </c>
       <c r="O53" s="9" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="P53" s="9" t="s">
         <v>26</v>
       </c>
       <c r="Q53" s="9"/>
       <c r="R53" s="9"/>
-      <c r="S53" s="9"/>
+      <c r="S53" s="9">
+        <v>1</v>
+      </c>
       <c r="T53" s="9"/>
-      <c r="U53" s="9"/>
+      <c r="U53" s="11" t="s">
+        <v>32</v>
+      </c>
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B54" s="5">
         <v>46073.71759134259</v>
       </c>
-      <c r="C54" s="6"/>
+      <c r="C54" s="5">
+        <v>46191.7899369213</v>
+      </c>
       <c r="D54" s="5">
-        <v>46129.782612256946</v>
+        <v>46191.7899528125</v>
       </c>
       <c r="E54" s="6" t="s">
+        <v>199</v>
+      </c>
+      <c r="F54" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="G54" s="6" t="s">
         <v>200</v>
       </c>
-      <c r="F54" s="6" t="s">
-        <v>26</v>
-      </c>
-      <c r="G54" s="6" t="s">
+      <c r="H54" s="6" t="s">
         <v>201</v>
-      </c>
-      <c r="H54" s="6" t="s">
-        <v>202</v>
       </c>
       <c r="I54" s="5">
         <v>46073</v>
@@ -4588,13 +4606,13 @@
         <v>26</v>
       </c>
       <c r="N54" s="6" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="O54" s="6" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="P54" s="6" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="Q54" s="5">
         <v>46073</v>
@@ -4603,37 +4621,39 @@
         <v>46083</v>
       </c>
       <c r="S54" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T54" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="U54" s="10" t="s">
-        <v>56</v>
+      <c r="U54" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="55" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A55" s="7" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B55" s="8">
         <v>46073.71759157407</v>
       </c>
-      <c r="C55" s="9"/>
+      <c r="C55" s="8">
+        <v>46191.79035826389</v>
+      </c>
       <c r="D55" s="8">
-        <v>46154.0951240162</v>
+        <v>46191.790375833334</v>
       </c>
       <c r="E55" s="9" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="F55" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G55" s="9" t="s">
+        <v>200</v>
+      </c>
+      <c r="H55" s="9" t="s">
         <v>201</v>
-      </c>
-      <c r="H55" s="9" t="s">
-        <v>202</v>
       </c>
       <c r="I55" s="8">
         <v>46084</v>
@@ -4651,13 +4671,13 @@
         <v>26</v>
       </c>
       <c r="N55" s="9" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="O55" s="9" t="s">
+        <v>205</v>
+      </c>
+      <c r="P55" s="9" t="s">
         <v>206</v>
-      </c>
-      <c r="P55" s="9" t="s">
-        <v>207</v>
       </c>
       <c r="Q55" s="8">
         <v>46084</v>
@@ -4666,37 +4686,39 @@
         <v>46101</v>
       </c>
       <c r="S55" s="9">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T55" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="U55" s="10" t="s">
-        <v>56</v>
+      <c r="U55" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="56" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B56" s="5">
         <v>46073.71759181713</v>
       </c>
-      <c r="C56" s="6"/>
+      <c r="C56" s="5">
+        <v>46191.789681423616</v>
+      </c>
       <c r="D56" s="5">
-        <v>46154.09512475695</v>
+        <v>46191.79037549769</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="F56" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G56" s="6" t="s">
+        <v>192</v>
+      </c>
+      <c r="H56" s="6" t="s">
         <v>193</v>
-      </c>
-      <c r="H56" s="6" t="s">
-        <v>194</v>
       </c>
       <c r="I56" s="5">
         <v>46104</v>
@@ -4714,13 +4736,13 @@
         <v>26</v>
       </c>
       <c r="N56" s="6" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="O56" s="6" t="s">
+        <v>209</v>
+      </c>
+      <c r="P56" s="6" t="s">
         <v>210</v>
-      </c>
-      <c r="P56" s="6" t="s">
-        <v>211</v>
       </c>
       <c r="Q56" s="5">
         <v>46104</v>
@@ -4729,13 +4751,13 @@
         <v>46105</v>
       </c>
       <c r="S56" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T56" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="U56" s="10" t="s">
-        <v>56</v>
+      <c r="U56" s="12" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.25">
@@ -4747,7 +4769,7 @@
       </c>
       <c r="C57" s="9"/>
       <c r="D57" s="8">
-        <v>46083.66877225695</v>
+        <v>46191.7884132176</v>
       </c>
       <c r="E57" s="9" t="s">
         <v>184</v>
@@ -4845,7 +4867,7 @@
         <v>31</v>
       </c>
       <c r="U58" s="12" t="s">
-        <v>190</v>
+        <v>211</v>
       </c>
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.25">
@@ -4908,7 +4930,7 @@
         <v>31</v>
       </c>
       <c r="U59" s="12" t="s">
-        <v>190</v>
+        <v>211</v>
       </c>
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.25">
@@ -4971,7 +4993,7 @@
         <v>31</v>
       </c>
       <c r="U60" s="12" t="s">
-        <v>190</v>
+        <v>211</v>
       </c>
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.25">
@@ -5097,7 +5119,7 @@
         <v>228</v>
       </c>
       <c r="U62" s="12" t="s">
-        <v>190</v>
+        <v>211</v>
       </c>
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.25">
@@ -5156,7 +5178,7 @@
       </c>
       <c r="C64" s="6"/>
       <c r="D64" s="5">
-        <v>46126.195007222224</v>
+        <v>46191.78969853009</v>
       </c>
       <c r="E64" s="6" t="s">
         <v>233</v>
@@ -5189,7 +5211,7 @@
         <v>230</v>
       </c>
       <c r="O64" s="6" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="P64" s="6" t="s">
         <v>234</v>
@@ -5206,8 +5228,8 @@
       <c r="T64" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="U64" s="10" t="s">
-        <v>56</v>
+      <c r="U64" s="12" t="s">
+        <v>211</v>
       </c>
     </row>
     <row r="65" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Actualiza portafolio 2026-06-18 21:34 UTC
</commit_message>
<xml_diff>
--- a/data/50001498 - CALABRESSE METRO STO DOMINGO POZOS.xlsx
+++ b/data/50001498 - CALABRESSE METRO STO DOMINGO POZOS.xlsx
@@ -11,7 +11,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1004" uniqueCount="289">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1005" uniqueCount="289">
   <si>
     <t xml:space="preserve">50001498-CALABRESSE METRO STO DOMINGO  POZOS  </t>
   </si>
@@ -319,6 +319,9 @@
     <t>Alabe,Tablero OT 4201,rodete OT 4200,Motor,Sensores,Materiales a codigo // compras locales aprovisionamientomiento:OT  4200</t>
   </si>
   <si>
+    <t>Tarea en curso</t>
+  </si>
+  <si>
     <t>1213380470331424</t>
   </si>
   <si>
@@ -644,9 +647,6 @@
   </si>
   <si>
     <t>Fabricación externa ,Revestimiento</t>
-  </si>
-  <si>
-    <t>Tarea en curso</t>
   </si>
   <si>
     <t>1213380470331441</t>
@@ -2799,7 +2799,7 @@
       </c>
       <c r="C25" s="9"/>
       <c r="D25" s="8">
-        <v>46182.68306111111</v>
+        <v>46191.88830023148</v>
       </c>
       <c r="E25" s="9" t="s">
         <v>100</v>
@@ -2835,11 +2835,13 @@
       <c r="R25" s="9"/>
       <c r="S25" s="9"/>
       <c r="T25" s="9"/>
-      <c r="U25" s="9"/>
+      <c r="U25" s="12" t="s">
+        <v>102</v>
+      </c>
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" s="4" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="B26" s="5">
         <v>46073.7175902662</v>
@@ -2851,16 +2853,16 @@
         <v>46155.86710392361</v>
       </c>
       <c r="E26" s="6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="F26" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G26" s="6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H26" s="6" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="I26" s="5">
         <v>46006</v>
@@ -2881,7 +2883,7 @@
         <v>100</v>
       </c>
       <c r="O26" s="6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="P26" s="6" t="s">
         <v>100</v>
@@ -2904,7 +2906,7 @@
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" s="7" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="B27" s="8">
         <v>46073.7175905787</v>
@@ -2916,16 +2918,16 @@
         <v>46097.52605688658</v>
       </c>
       <c r="E27" s="9" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="F27" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G27" s="9" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H27" s="9" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="I27" s="8">
         <v>46006</v>
@@ -2943,13 +2945,13 @@
         <v>26</v>
       </c>
       <c r="N27" s="9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="O27" s="9" t="s">
         <v>79</v>
       </c>
       <c r="P27" s="9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="Q27" s="9"/>
       <c r="R27" s="9"/>
@@ -2957,7 +2959,7 @@
         <v>0</v>
       </c>
       <c r="T27" s="11" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="U27" s="10" t="s">
         <v>56</v>
@@ -2965,7 +2967,7 @@
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" s="4" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="B28" s="5">
         <v>46073.71759086805</v>
@@ -2977,16 +2979,16 @@
         <v>46155.866878229164</v>
       </c>
       <c r="E28" s="6" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="F28" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G28" s="6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H28" s="6" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="I28" s="5">
         <v>46027</v>
@@ -3004,13 +3006,13 @@
         <v>26</v>
       </c>
       <c r="N28" s="6" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="O28" s="6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="P28" s="6" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="Q28" s="6"/>
       <c r="R28" s="6"/>
@@ -3018,7 +3020,7 @@
         <v>0</v>
       </c>
       <c r="T28" s="11" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="U28" s="10" t="s">
         <v>56</v>
@@ -3026,7 +3028,7 @@
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" s="7" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="B29" s="8">
         <v>46073.71759118055</v>
@@ -3038,16 +3040,16 @@
         <v>46128.63717174769</v>
       </c>
       <c r="E29" s="9" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F29" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G29" s="9" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H29" s="9" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="I29" s="8">
         <v>46027</v>
@@ -3065,13 +3067,13 @@
         <v>26</v>
       </c>
       <c r="N29" s="9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="O29" s="9" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="P29" s="9" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="Q29" s="9"/>
       <c r="R29" s="9"/>
@@ -3079,7 +3081,7 @@
         <v>0</v>
       </c>
       <c r="T29" s="11" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="U29" s="10" t="s">
         <v>56</v>
@@ -3087,7 +3089,7 @@
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" s="4" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="B30" s="5">
         <v>46073.7175909838</v>
@@ -3099,16 +3101,16 @@
         <v>46155.90358277778</v>
       </c>
       <c r="E30" s="6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F30" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G30" s="6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H30" s="6" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="I30" s="5">
         <v>46013</v>
@@ -3129,7 +3131,7 @@
         <v>100</v>
       </c>
       <c r="O30" s="6" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="P30" s="6" t="s">
         <v>100</v>
@@ -3152,7 +3154,7 @@
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31" s="7" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="B31" s="8">
         <v>46073.71759126158</v>
@@ -3164,16 +3166,16 @@
         <v>46097.52608802084</v>
       </c>
       <c r="E31" s="9" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="F31" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G31" s="9" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H31" s="9" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="I31" s="8">
         <v>46013</v>
@@ -3191,13 +3193,13 @@
         <v>26</v>
       </c>
       <c r="N31" s="9" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="O31" s="9" t="s">
         <v>82</v>
       </c>
       <c r="P31" s="9" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="Q31" s="9"/>
       <c r="R31" s="9"/>
@@ -3205,7 +3207,7 @@
         <v>0</v>
       </c>
       <c r="T31" s="11" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="U31" s="10" t="s">
         <v>56</v>
@@ -3213,7 +3215,7 @@
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A32" s="4" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="B32" s="5">
         <v>46073.71759153935</v>
@@ -3225,16 +3227,16 @@
         <v>46155.90355751157</v>
       </c>
       <c r="E32" s="6" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="F32" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G32" s="6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H32" s="6" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="I32" s="5">
         <v>46017</v>
@@ -3252,13 +3254,13 @@
         <v>26</v>
       </c>
       <c r="N32" s="6" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="O32" s="6" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="P32" s="6" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="Q32" s="6"/>
       <c r="R32" s="6"/>
@@ -3266,7 +3268,7 @@
         <v>0</v>
       </c>
       <c r="T32" s="11" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="U32" s="10" t="s">
         <v>56</v>
@@ -3274,7 +3276,7 @@
     </row>
     <row r="33" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A33" s="7" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="B33" s="8">
         <v>46073.717592685185</v>
@@ -3286,16 +3288,16 @@
         <v>46182.683057222224</v>
       </c>
       <c r="E33" s="9" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="F33" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G33" s="9" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H33" s="9" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="I33" s="8">
         <v>46013</v>
@@ -3316,7 +3318,7 @@
         <v>100</v>
       </c>
       <c r="O33" s="9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="P33" s="9" t="s">
         <v>100</v>
@@ -3339,7 +3341,7 @@
     </row>
     <row r="34" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A34" s="4" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="B34" s="5">
         <v>46073.71759302083</v>
@@ -3351,16 +3353,16 @@
         <v>46182.6827475</v>
       </c>
       <c r="E34" s="6" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="F34" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G34" s="6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H34" s="6" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="I34" s="5">
         <v>46013</v>
@@ -3378,13 +3380,13 @@
         <v>26</v>
       </c>
       <c r="N34" s="6" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="O34" s="6" t="s">
         <v>85</v>
       </c>
       <c r="P34" s="6" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="Q34" s="6"/>
       <c r="R34" s="6"/>
@@ -3392,7 +3394,7 @@
         <v>0</v>
       </c>
       <c r="T34" s="11" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="U34" s="10" t="s">
         <v>56</v>
@@ -3400,7 +3402,7 @@
     </row>
     <row r="35" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A35" s="7" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="B35" s="8">
         <v>46073.71758986111</v>
@@ -3412,16 +3414,16 @@
         <v>46182.682943541666</v>
       </c>
       <c r="E35" s="9" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="F35" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G35" s="9" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H35" s="9" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="I35" s="8">
         <v>46017</v>
@@ -3439,13 +3441,13 @@
         <v>26</v>
       </c>
       <c r="N35" s="9" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="O35" s="9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="P35" s="9" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="Q35" s="9"/>
       <c r="R35" s="9"/>
@@ -3453,7 +3455,7 @@
         <v>0</v>
       </c>
       <c r="T35" s="11" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="U35" s="10" t="s">
         <v>56</v>
@@ -3461,26 +3463,28 @@
     </row>
     <row r="36" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A36" s="4" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B36" s="5">
         <v>46073.7175918287</v>
       </c>
-      <c r="C36" s="6"/>
+      <c r="C36" s="5">
+        <v>46191.888280127314</v>
+      </c>
       <c r="D36" s="5">
-        <v>46169.843397372686</v>
+        <v>46191.89070638889</v>
       </c>
       <c r="E36" s="6" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="F36" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G36" s="6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H36" s="6" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="I36" s="5">
         <v>46007</v>
@@ -3501,7 +3505,7 @@
         <v>100</v>
       </c>
       <c r="O36" s="6" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="P36" s="6" t="s">
         <v>100</v>
@@ -3513,18 +3517,18 @@
         <v>46114</v>
       </c>
       <c r="S36" s="6">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="T36" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="U36" s="10" t="s">
-        <v>56</v>
+      <c r="U36" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="37" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A37" s="7" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="B37" s="8">
         <v>46073.71759209491</v>
@@ -3536,16 +3540,16 @@
         <v>46169.84329747685</v>
       </c>
       <c r="E37" s="9" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="F37" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G37" s="9" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H37" s="9" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="I37" s="8">
         <v>46007</v>
@@ -3563,13 +3567,13 @@
         <v>26</v>
       </c>
       <c r="N37" s="9" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="O37" s="9" t="s">
         <v>89</v>
       </c>
       <c r="P37" s="9" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="Q37" s="9"/>
       <c r="R37" s="9"/>
@@ -3577,7 +3581,7 @@
         <v>0</v>
       </c>
       <c r="T37" s="11" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="U37" s="10" t="s">
         <v>56</v>
@@ -3585,26 +3589,26 @@
     </row>
     <row r="38" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A38" s="4" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="B38" s="5">
         <v>46073.71759234954</v>
       </c>
       <c r="C38" s="6"/>
       <c r="D38" s="5">
-        <v>46183.686308344906</v>
+        <v>46191.88833190972</v>
       </c>
       <c r="E38" s="6" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="F38" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G38" s="6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="H38" s="6" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="I38" s="5">
         <v>46017</v>
@@ -3622,13 +3626,13 @@
         <v>26</v>
       </c>
       <c r="N38" s="6" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="O38" s="6" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="P38" s="6" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="Q38" s="6"/>
       <c r="R38" s="6"/>
@@ -3636,7 +3640,7 @@
         <v>0</v>
       </c>
       <c r="T38" s="11" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="U38" s="10" t="s">
         <v>56</v>
@@ -3644,7 +3648,7 @@
     </row>
     <row r="39" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A39" s="7" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="B39" s="8">
         <v>46076.59415034722</v>
@@ -3656,16 +3660,16 @@
         <v>46156.618615775464</v>
       </c>
       <c r="E39" s="9" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="F39" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G39" s="9" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="H39" s="9" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="I39" s="8">
         <v>46013</v>
@@ -3686,7 +3690,7 @@
         <v>100</v>
       </c>
       <c r="O39" s="9" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="P39" s="9" t="s">
         <v>100</v>
@@ -3709,7 +3713,7 @@
     </row>
     <row r="40" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A40" s="4" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="B40" s="5">
         <v>46076.59428157407</v>
@@ -3721,16 +3725,16 @@
         <v>46154.86737356482</v>
       </c>
       <c r="E40" s="6" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="F40" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G40" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="H40" s="6" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="I40" s="5">
         <v>46013</v>
@@ -3748,13 +3752,13 @@
         <v>26</v>
       </c>
       <c r="N40" s="6" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="O40" s="6" t="s">
         <v>92</v>
       </c>
       <c r="P40" s="6" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="Q40" s="5">
         <v>46013</v>
@@ -3766,7 +3770,7 @@
         <v>0</v>
       </c>
       <c r="T40" s="11" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="U40" s="10" t="s">
         <v>56</v>
@@ -3774,7 +3778,7 @@
     </row>
     <row r="41" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A41" s="7" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="B41" s="8">
         <v>46076.59448399306</v>
@@ -3786,16 +3790,16 @@
         <v>46154.86810545139</v>
       </c>
       <c r="E41" s="9" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="F41" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G41" s="9" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="H41" s="9" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="I41" s="8">
         <v>46057</v>
@@ -3813,13 +3817,13 @@
         <v>26</v>
       </c>
       <c r="N41" s="9" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="O41" s="9" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="P41" s="9" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="Q41" s="8">
         <v>46057</v>
@@ -3831,7 +3835,7 @@
         <v>0</v>
       </c>
       <c r="T41" s="11" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="U41" s="10" t="s">
         <v>56</v>
@@ -3839,7 +3843,7 @@
     </row>
     <row r="42" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A42" s="4" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="B42" s="5">
         <v>46073.71759148148</v>
@@ -3851,16 +3855,16 @@
         <v>46182.53063152778</v>
       </c>
       <c r="E42" s="6" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="F42" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G42" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="H42" s="6" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="I42" s="5">
         <v>46013</v>
@@ -3881,7 +3885,7 @@
         <v>100</v>
       </c>
       <c r="O42" s="6" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="P42" s="6" t="s">
         <v>100</v>
@@ -3904,7 +3908,7 @@
     </row>
     <row r="43" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A43" s="7" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="B43" s="8">
         <v>46073.717591759254</v>
@@ -3916,16 +3920,16 @@
         <v>46182.53047055556</v>
       </c>
       <c r="E43" s="9" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="F43" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G43" s="9" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="H43" s="9" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="I43" s="8">
         <v>46013</v>
@@ -3943,13 +3947,13 @@
         <v>26</v>
       </c>
       <c r="N43" s="9" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="O43" s="9" t="s">
         <v>95</v>
       </c>
       <c r="P43" s="9" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="Q43" s="9"/>
       <c r="R43" s="9"/>
@@ -3957,7 +3961,7 @@
         <v>0</v>
       </c>
       <c r="T43" s="11" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="U43" s="10" t="s">
         <v>56</v>
@@ -3965,7 +3969,7 @@
     </row>
     <row r="44" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A44" s="4" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="B44" s="5">
         <v>46073.71759204861</v>
@@ -3977,16 +3981,16 @@
         <v>46182.53060627315</v>
       </c>
       <c r="E44" s="6" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="F44" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G44" s="6" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="H44" s="6" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="I44" s="5">
         <v>46037</v>
@@ -4004,13 +4008,13 @@
         <v>26</v>
       </c>
       <c r="N44" s="6" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="O44" s="6" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="P44" s="6" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="Q44" s="6"/>
       <c r="R44" s="6"/>
@@ -4018,7 +4022,7 @@
         <v>0</v>
       </c>
       <c r="T44" s="11" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="U44" s="10" t="s">
         <v>56</v>
@@ -4026,7 +4030,7 @@
     </row>
     <row r="45" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A45" s="7" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
       <c r="B45" s="8">
         <v>46073.71759234954</v>
@@ -4036,7 +4040,7 @@
         <v>46156.618706249996</v>
       </c>
       <c r="E45" s="9" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="F45" s="9" t="s">
         <v>25</v>
@@ -4060,7 +4064,7 @@
         <v>26</v>
       </c>
       <c r="O45" s="9" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="P45" s="9" t="s">
         <v>26</v>
@@ -4073,7 +4077,7 @@
     </row>
     <row r="46" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A46" s="4" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
       <c r="B46" s="5">
         <v>46073.717592615736</v>
@@ -4085,16 +4089,16 @@
         <v>46154.09504209491</v>
       </c>
       <c r="E46" s="6" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="F46" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G46" s="6" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="H46" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="I46" s="5">
         <v>46009</v>
@@ -4112,13 +4116,13 @@
         <v>26</v>
       </c>
       <c r="N46" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="O46" s="6" t="s">
         <v>69</v>
       </c>
       <c r="P46" s="6" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="Q46" s="5">
         <v>46009</v>
@@ -4138,7 +4142,7 @@
     </row>
     <row r="47" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A47" s="7" t="s">
-        <v>172</v>
+        <v>173</v>
       </c>
       <c r="B47" s="8">
         <v>46073.71758997685</v>
@@ -4150,16 +4154,16 @@
         <v>46154.09509461805</v>
       </c>
       <c r="E47" s="9" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="F47" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G47" s="9" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="H47" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="I47" s="8">
         <v>46065</v>
@@ -4177,13 +4181,13 @@
         <v>26</v>
       </c>
       <c r="N47" s="9" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="O47" s="9" t="s">
-        <v>174</v>
+        <v>175</v>
       </c>
       <c r="P47" s="9" t="s">
-        <v>175</v>
+        <v>176</v>
       </c>
       <c r="Q47" s="8">
         <v>46065</v>
@@ -4203,7 +4207,7 @@
     </row>
     <row r="48" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A48" s="4" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="B48" s="5">
         <v>46091.72801988426</v>
@@ -4215,16 +4219,16 @@
         <v>46154.09513386574</v>
       </c>
       <c r="E48" s="6" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F48" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G48" s="6" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="H48" s="6" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="I48" s="5">
         <v>46072</v>
@@ -4242,13 +4246,13 @@
         <v>26</v>
       </c>
       <c r="N48" s="6" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="O48" s="6" t="s">
-        <v>173</v>
+        <v>174</v>
       </c>
       <c r="P48" s="6" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="Q48" s="5">
         <v>46072</v>
@@ -4268,7 +4272,7 @@
     </row>
     <row r="49" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A49" s="7" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="B49" s="8">
         <v>46091.728057939814</v>
@@ -4278,16 +4282,16 @@
         <v>46161.2013843287</v>
       </c>
       <c r="E49" s="9" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F49" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G49" s="9" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
       <c r="H49" s="9" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="I49" s="8">
         <v>46160</v>
@@ -4305,13 +4309,13 @@
         <v>26</v>
       </c>
       <c r="N49" s="9" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
       <c r="O49" s="9" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="P49" s="9" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="Q49" s="8">
         <v>46160</v>
@@ -4331,7 +4335,7 @@
     </row>
     <row r="50" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A50" s="4" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="B50" s="5">
         <v>46073.71759030093</v>
@@ -4343,7 +4347,7 @@
         <v>46191.789304328704</v>
       </c>
       <c r="E50" s="6" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F50" s="6" t="s">
         <v>25</v>
@@ -4367,7 +4371,7 @@
         <v>26</v>
       </c>
       <c r="O50" s="6" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="P50" s="6" t="s">
         <v>26</v>
@@ -4384,7 +4388,7 @@
     </row>
     <row r="51" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A51" s="7" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="B51" s="8">
         <v>46073.7175905787</v>
@@ -4396,16 +4400,16 @@
         <v>46191.788422488426</v>
       </c>
       <c r="E51" s="9" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="F51" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G51" s="9" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="H51" s="9" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="I51" s="8">
         <v>46069</v>
@@ -4423,13 +4427,13 @@
         <v>26</v>
       </c>
       <c r="N51" s="9" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="O51" s="9" t="s">
-        <v>162</v>
+        <v>163</v>
       </c>
       <c r="P51" s="9" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="Q51" s="8">
         <v>46069</v>
@@ -4449,7 +4453,7 @@
     </row>
     <row r="52" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A52" s="4" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="B52" s="5">
         <v>46073.717590810185</v>
@@ -4461,16 +4465,16 @@
         <v>46191.789293194444</v>
       </c>
       <c r="E52" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F52" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G52" s="6" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="H52" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="I52" s="5">
         <v>46071</v>
@@ -4488,13 +4492,13 @@
         <v>26</v>
       </c>
       <c r="N52" s="6" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="O52" s="6" t="s">
-        <v>163</v>
+        <v>164</v>
       </c>
       <c r="P52" s="6" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="Q52" s="5">
         <v>46071</v>
@@ -4514,7 +4518,7 @@
     </row>
     <row r="53" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A53" s="7" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B53" s="8">
         <v>46073.717591099536</v>
@@ -4526,7 +4530,7 @@
         <v>46191.79038505787</v>
       </c>
       <c r="E53" s="9" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="F53" s="9" t="s">
         <v>25</v>
@@ -4550,7 +4554,7 @@
         <v>26</v>
       </c>
       <c r="O53" s="9" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="P53" s="9" t="s">
         <v>26</v>
@@ -4567,7 +4571,7 @@
     </row>
     <row r="54" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A54" s="4" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="B54" s="5">
         <v>46073.71759134259</v>
@@ -4579,16 +4583,16 @@
         <v>46191.7899528125</v>
       </c>
       <c r="E54" s="6" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="F54" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G54" s="6" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="H54" s="6" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="I54" s="5">
         <v>46073</v>
@@ -4606,13 +4610,13 @@
         <v>26</v>
       </c>
       <c r="N54" s="6" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="O54" s="6" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="P54" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="Q54" s="5">
         <v>46073</v>
@@ -4632,7 +4636,7 @@
     </row>
     <row r="55" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A55" s="7" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="B55" s="8">
         <v>46073.71759157407</v>
@@ -4644,16 +4648,16 @@
         <v>46191.790375833334</v>
       </c>
       <c r="E55" s="9" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="F55" s="9" t="s">
         <v>26</v>
       </c>
       <c r="G55" s="9" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="H55" s="9" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="I55" s="8">
         <v>46084</v>
@@ -4671,13 +4675,13 @@
         <v>26</v>
       </c>
       <c r="N55" s="9" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="O55" s="9" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="P55" s="9" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="Q55" s="8">
         <v>46084</v>
@@ -4697,7 +4701,7 @@
     </row>
     <row r="56" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A56" s="4" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="B56" s="5">
         <v>46073.71759181713</v>
@@ -4709,16 +4713,16 @@
         <v>46191.79037549769</v>
       </c>
       <c r="E56" s="6" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="F56" s="6" t="s">
         <v>26</v>
       </c>
       <c r="G56" s="6" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
       <c r="H56" s="6" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="I56" s="5">
         <v>46104</v>
@@ -4736,13 +4740,13 @@
         <v>26</v>
       </c>
       <c r="N56" s="6" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="O56" s="6" t="s">
-        <v>209</v>
+        <v>210</v>
       </c>
       <c r="P56" s="6" t="s">
-        <v>210</v>
+        <v>211</v>
       </c>
       <c r="Q56" s="5">
         <v>46104</v>
@@ -4757,7 +4761,7 @@
         <v>31</v>
       </c>
       <c r="U56" s="12" t="s">
-        <v>211</v>
+        <v>102</v>
       </c>
     </row>
     <row r="57" spans="1:21" x14ac:dyDescent="0.25">
@@ -4772,7 +4776,7 @@
         <v>46191.7884132176</v>
       </c>
       <c r="E57" s="9" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F57" s="9" t="s">
         <v>25</v>
@@ -4825,10 +4829,10 @@
         <v>26</v>
       </c>
       <c r="G58" s="6" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="H58" s="6" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="I58" s="5">
         <v>46153</v>
@@ -4846,10 +4850,10 @@
         <v>26</v>
       </c>
       <c r="N58" s="6" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="O58" s="6" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="P58" s="6" t="s">
         <v>216</v>
@@ -4867,7 +4871,7 @@
         <v>31</v>
       </c>
       <c r="U58" s="12" t="s">
-        <v>211</v>
+        <v>102</v>
       </c>
     </row>
     <row r="59" spans="1:21" x14ac:dyDescent="0.25">
@@ -4888,10 +4892,10 @@
         <v>26</v>
       </c>
       <c r="G59" s="9" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="H59" s="9" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="I59" s="8">
         <v>46135</v>
@@ -4909,10 +4913,10 @@
         <v>26</v>
       </c>
       <c r="N59" s="9" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="O59" s="9" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="P59" s="9" t="s">
         <v>219</v>
@@ -4930,7 +4934,7 @@
         <v>31</v>
       </c>
       <c r="U59" s="12" t="s">
-        <v>211</v>
+        <v>102</v>
       </c>
     </row>
     <row r="60" spans="1:21" x14ac:dyDescent="0.25">
@@ -4951,10 +4955,10 @@
         <v>26</v>
       </c>
       <c r="G60" s="6" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="H60" s="6" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="I60" s="5">
         <v>46071</v>
@@ -4972,10 +4976,10 @@
         <v>26</v>
       </c>
       <c r="N60" s="6" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="O60" s="6" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="P60" s="6" t="s">
         <v>222</v>
@@ -4993,7 +4997,7 @@
         <v>31</v>
       </c>
       <c r="U60" s="12" t="s">
-        <v>211</v>
+        <v>102</v>
       </c>
     </row>
     <row r="61" spans="1:21" x14ac:dyDescent="0.25">
@@ -5005,7 +5009,7 @@
       </c>
       <c r="C61" s="9"/>
       <c r="D61" s="8">
-        <v>46119.188054259255</v>
+        <v>46191.88833803241</v>
       </c>
       <c r="E61" s="9" t="s">
         <v>54</v>
@@ -5014,10 +5018,10 @@
         <v>26</v>
       </c>
       <c r="G61" s="9" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="H61" s="9" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="I61" s="8">
         <v>46115</v>
@@ -5035,10 +5039,10 @@
         <v>26</v>
       </c>
       <c r="N61" s="9" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="O61" s="9" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="P61" s="9" t="s">
         <v>224</v>
@@ -5055,8 +5059,8 @@
       <c r="T61" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="U61" s="10" t="s">
-        <v>56</v>
+      <c r="U61" s="12" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="62" spans="1:21" x14ac:dyDescent="0.25">
@@ -5077,10 +5081,10 @@
         <v>26</v>
       </c>
       <c r="G62" s="6" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="H62" s="6" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="I62" s="5">
         <v>46139</v>
@@ -5098,10 +5102,10 @@
         <v>26</v>
       </c>
       <c r="N62" s="6" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="O62" s="6" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="P62" s="6" t="s">
         <v>227</v>
@@ -5119,7 +5123,7 @@
         <v>228</v>
       </c>
       <c r="U62" s="12" t="s">
-        <v>211</v>
+        <v>102</v>
       </c>
     </row>
     <row r="63" spans="1:21" x14ac:dyDescent="0.25">
@@ -5211,7 +5215,7 @@
         <v>230</v>
       </c>
       <c r="O64" s="6" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="P64" s="6" t="s">
         <v>234</v>
@@ -5229,7 +5233,7 @@
         <v>31</v>
       </c>
       <c r="U64" s="12" t="s">
-        <v>211</v>
+        <v>102</v>
       </c>
     </row>
     <row r="65" spans="1:21" x14ac:dyDescent="0.25">
@@ -5496,7 +5500,7 @@
         <v>46158.18178945602</v>
       </c>
       <c r="E69" s="9" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F69" s="9" t="s">
         <v>26</v>
@@ -5559,7 +5563,7 @@
         <v>46162.1685475</v>
       </c>
       <c r="E70" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F70" s="6" t="s">
         <v>26</v>
@@ -5589,7 +5593,7 @@
         <v>230</v>
       </c>
       <c r="O70" s="6" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="P70" s="6" t="s">
         <v>252</v>
@@ -5699,7 +5703,7 @@
         <v>254</v>
       </c>
       <c r="O72" s="6" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="P72" s="6" t="s">
         <v>258</v>
@@ -5954,7 +5958,7 @@
         <v>0</v>
       </c>
       <c r="T76" s="11" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="U76" s="10" t="s">
         <v>56</v>
@@ -6133,7 +6137,7 @@
         <v>0</v>
       </c>
       <c r="T79" s="11" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="U79" s="10" t="s">
         <v>56</v>

</xml_diff>

<commit_message>
KPI actualizado 2026-07-07 20:27 UTC
</commit_message>
<xml_diff>
--- a/data/50001498 - CALABRESSE METRO STO DOMINGO POZOS.xlsx
+++ b/data/50001498 - CALABRESSE METRO STO DOMINGO POZOS.xlsx
@@ -5281,7 +5281,7 @@
         <v>46193.60739422454</v>
       </c>
       <c r="D65" s="8">
-        <v>46195.608936585646</v>
+        <v>46210.82564115741</v>
       </c>
       <c r="E65" s="9" t="s">
         <v>238</v>
@@ -5331,8 +5331,8 @@
       <c r="T65" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="U65" s="12" t="s">
-        <v>213</v>
+      <c r="U65" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="66" spans="1:21" x14ac:dyDescent="0.25">
@@ -5346,7 +5346,7 @@
         <v>46193.60745574074</v>
       </c>
       <c r="D66" s="5">
-        <v>46195.60911005787</v>
+        <v>46210.825641759264</v>
       </c>
       <c r="E66" s="6" t="s">
         <v>242</v>
@@ -5396,8 +5396,8 @@
       <c r="T66" s="12" t="s">
         <v>230</v>
       </c>
-      <c r="U66" s="12" t="s">
-        <v>213</v>
+      <c r="U66" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="67" spans="1:21" x14ac:dyDescent="0.25">
@@ -5411,7 +5411,7 @@
         <v>46193.607493668984</v>
       </c>
       <c r="D67" s="8">
-        <v>46198.82799127315</v>
+        <v>46210.82564222222</v>
       </c>
       <c r="E67" s="9" t="s">
         <v>246</v>
@@ -5461,8 +5461,8 @@
       <c r="T67" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="U67" s="12" t="s">
-        <v>213</v>
+      <c r="U67" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="68" spans="1:21" x14ac:dyDescent="0.25">
@@ -5476,7 +5476,7 @@
         <v>46193.60764289352</v>
       </c>
       <c r="D68" s="5">
-        <v>46198.82948185185</v>
+        <v>46210.82564268519</v>
       </c>
       <c r="E68" s="6" t="s">
         <v>229</v>
@@ -5526,8 +5526,8 @@
       <c r="T68" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="U68" s="12" t="s">
-        <v>213</v>
+      <c r="U68" s="11" t="s">
+        <v>32</v>
       </c>
     </row>
     <row r="69" spans="1:21" x14ac:dyDescent="0.25">

</xml_diff>

<commit_message>
Actualiza portafolio 2026-08-13 16:59 UTC
</commit_message>
<xml_diff>
--- a/data/50001498 - CALABRESSE METRO STO DOMINGO POZOS.xlsx
+++ b/data/50001498 - CALABRESSE METRO STO DOMINGO POZOS.xlsx
@@ -5729,9 +5729,11 @@
       <c r="B72" s="5">
         <v>46073.71759042824</v>
       </c>
-      <c r="C72" s="6"/>
+      <c r="C72" s="5">
+        <v>46247.63130804399</v>
+      </c>
       <c r="D72" s="5">
-        <v>46246.81082678241</v>
+        <v>46247.63131010417</v>
       </c>
       <c r="E72" s="6" t="s">
         <v>259</v>

</xml_diff>